<commit_message>
Customer Sales report almost done also pickup weight bug fixed
</commit_message>
<xml_diff>
--- a/public/reports/customer_sales_report.xlsx
+++ b/public/reports/customer_sales_report.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="15">
   <si>
     <t>Origin</t>
   </si>
@@ -23,70 +23,43 @@
     <t>Client Name</t>
   </si>
   <si>
-    <t>Multiple</t>
-  </si>
-  <si>
-    <t>Abbottabad</t>
-  </si>
-  <si>
-    <t>Abdul Hakim</t>
-  </si>
-  <si>
-    <t>Ahmed Pur East</t>
-  </si>
-  <si>
-    <t>Alipur</t>
-  </si>
-  <si>
-    <t>Ali Pur Chatta</t>
-  </si>
-  <si>
-    <t>Arifwala</t>
-  </si>
-  <si>
-    <t>Attock</t>
-  </si>
-  <si>
-    <t>Badin</t>
-  </si>
-  <si>
-    <t>Bahawalnagar</t>
-  </si>
-  <si>
-    <t>Bahawalpur</t>
-  </si>
-  <si>
-    <t>Islamabad</t>
+    <t>February 2018</t>
+  </si>
+  <si>
+    <t>March 2018</t>
+  </si>
+  <si>
+    <t>April 2018</t>
+  </si>
+  <si>
+    <t>May 2018</t>
+  </si>
+  <si>
+    <t>June 2018</t>
+  </si>
+  <si>
+    <t>July 2018</t>
+  </si>
+  <si>
+    <t>August 2018</t>
+  </si>
+  <si>
+    <t>Parcels</t>
+  </si>
+  <si>
+    <t>Weight</t>
+  </si>
+  <si>
+    <t>COD Amount</t>
+  </si>
+  <si>
+    <t>Revenue</t>
   </si>
   <si>
     <t>Karachi</t>
   </si>
   <si>
     <t>Farrell Ltd</t>
-  </si>
-  <si>
-    <t>Murphy PLC</t>
-  </si>
-  <si>
-    <t>Swift LLC</t>
-  </si>
-  <si>
-    <t>Stehr LLC</t>
-  </si>
-  <si>
-    <t>Bruen Inc</t>
-  </si>
-  <si>
-    <t>Mohr-Collier</t>
-  </si>
-  <si>
-    <t>Torp, Stamm and Wilkinson</t>
-  </si>
-  <si>
-    <t>Lahore</t>
-  </si>
-  <si>
-    <t>Multan</t>
   </si>
 </sst>
 </file>
@@ -94,9 +67,18 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <b val="0"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b val="1"/>
       <i val="0"/>
       <strike val="0"/>
       <u val="none"/>
@@ -122,9 +104,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="1" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -425,127 +410,248 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:B25"/>
+  <dimension ref="A1:AD4"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+    <row r="1" spans="1:30">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+      <c r="O1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="P1" s="1"/>
+      <c r="Q1" s="1"/>
+      <c r="R1" s="1"/>
+      <c r="S1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="T1" s="1"/>
+      <c r="U1" s="1"/>
+      <c r="V1" s="1"/>
+      <c r="W1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="X1" s="1"/>
+      <c r="Y1" s="1"/>
+      <c r="Z1" s="1"/>
+      <c r="AA1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="AB1" s="1"/>
+      <c r="AC1" s="1"/>
+      <c r="AD1" s="1"/>
     </row>
-    <row r="4" spans="1:2">
-      <c r="A4" t="s">
-        <v>2</v>
+    <row r="2" spans="1:30">
+      <c r="C2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" t="s">
+        <v>9</v>
+      </c>
+      <c r="H2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I2" t="s">
+        <v>11</v>
+      </c>
+      <c r="J2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K2" t="s">
+        <v>9</v>
+      </c>
+      <c r="L2" t="s">
+        <v>10</v>
+      </c>
+      <c r="M2" t="s">
+        <v>11</v>
+      </c>
+      <c r="N2" t="s">
+        <v>12</v>
+      </c>
+      <c r="O2" t="s">
+        <v>9</v>
+      </c>
+      <c r="P2" t="s">
+        <v>10</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>11</v>
+      </c>
+      <c r="R2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S2" t="s">
+        <v>9</v>
+      </c>
+      <c r="T2" t="s">
+        <v>10</v>
+      </c>
+      <c r="U2" t="s">
+        <v>11</v>
+      </c>
+      <c r="V2" t="s">
+        <v>12</v>
+      </c>
+      <c r="W2" t="s">
+        <v>9</v>
+      </c>
+      <c r="X2" t="s">
+        <v>10</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>11</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>12</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>9</v>
+      </c>
+      <c r="AB2" t="s">
+        <v>10</v>
+      </c>
+      <c r="AC2" t="s">
+        <v>11</v>
+      </c>
+      <c r="AD2" t="s">
+        <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
-      <c r="A5" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2">
-      <c r="A6" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2">
-      <c r="A7" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2">
-      <c r="A8" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2">
-      <c r="A9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2">
-      <c r="A10" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2">
-      <c r="A11" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2">
-      <c r="A12" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2">
-      <c r="A13" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2">
-      <c r="A14" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2">
-      <c r="A15" t="s">
+    <row r="4" spans="1:30">
+      <c r="A4" s="1" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="16" spans="1:2">
-      <c r="A16" t="s">
+      <c r="B4" t="s">
         <v>14</v>
       </c>
-      <c r="B16" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2">
-      <c r="B17" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2">
-      <c r="B18" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2">
-      <c r="B19" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2">
-      <c r="B20" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2">
-      <c r="B21" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2">
-      <c r="B22" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2">
-      <c r="A24" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2">
-      <c r="A25" t="s">
-        <v>23</v>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="K4">
+        <v>0</v>
+      </c>
+      <c r="L4">
+        <v>0</v>
+      </c>
+      <c r="M4">
+        <v>0</v>
+      </c>
+      <c r="N4">
+        <v>0</v>
+      </c>
+      <c r="O4">
+        <v>0</v>
+      </c>
+      <c r="P4">
+        <v>0</v>
+      </c>
+      <c r="Q4">
+        <v>0</v>
+      </c>
+      <c r="R4">
+        <v>0</v>
+      </c>
+      <c r="S4">
+        <v>0</v>
+      </c>
+      <c r="T4">
+        <v>0</v>
+      </c>
+      <c r="U4">
+        <v>0</v>
+      </c>
+      <c r="V4">
+        <v>0</v>
+      </c>
+      <c r="W4">
+        <v>59</v>
+      </c>
+      <c r="X4">
+        <v>13</v>
+      </c>
+      <c r="Y4">
+        <v>205422</v>
+      </c>
+      <c r="Z4">
+        <v>0</v>
+      </c>
+      <c r="AA4">
+        <v>0</v>
+      </c>
+      <c r="AB4">
+        <v>0</v>
+      </c>
+      <c r="AC4">
+        <v>0</v>
+      </c>
+      <c r="AD4">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
   <sheetProtection sheet="false" objects="false" scenarios="false" formatCells="false" formatColumns="false" formatRows="false" insertColumns="false" insertRows="false" insertHyperlinks="false" deleteColumns="false" deleteRows="false" selectLockedCells="false" sort="false" autoFilter="false" pivotTables="false" selectUnlockedCells="false"/>
+  <mergeCells>
+    <mergeCell ref="C1:F1"/>
+    <mergeCell ref="G1:J1"/>
+    <mergeCell ref="K1:N1"/>
+    <mergeCell ref="O1:R1"/>
+    <mergeCell ref="S1:V1"/>
+    <mergeCell ref="W1:Z1"/>
+    <mergeCell ref="AA1:AD1"/>
+  </mergeCells>
   <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1"/>

</xml_diff>